<commit_message>
Add cleaned objective labels
</commit_message>
<xml_diff>
--- a/code/data_cleaning/annotations_summary_manually_edited.xlsx
+++ b/code/data_cleaning/annotations_summary_manually_edited.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\5298954\Documents\Github_Repos\GIMA_thesis\code\data_cleaning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB1C5612-09C6-49ED-8F1B-3A46DFC48E69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{399BBC61-2D36-4DE3-A9AD-2F6D739FF93B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28950" yWindow="3165" windowWidth="29040" windowHeight="15720" xr2:uid="{1CC9DFF3-CCD0-41B0-B0A8-07B4A468A7A4}"/>
+    <workbookView xWindow="28680" yWindow="-9540" windowWidth="29040" windowHeight="15720" xr2:uid="{1CC9DFF3-CCD0-41B0-B0A8-07B4A468A7A4}"/>
   </bookViews>
   <sheets>
     <sheet name="annotations_summary_manually_ed" sheetId="1" r:id="rId1"/>
@@ -21,14 +21,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="106">
   <si>
     <t>File</t>
   </si>
   <si>
-    <t>author</t>
-  </si>
-  <si>
     <t>"(1976_Boskamp_MJ_De_invloed_van_persoonskenmerken)";De invloed van persoonskenmerken op verschillende vormen van gebruik van een binnenstad';M.J. Boskamp';"Oktober ""(1976'",4,1976_Boskamp_MJ_De_invloed_van_persoonskenmerken,De invloed van persoonskenmerken op verschillende vormen van gebruik van een binnenstad,M.J. Boskamp,"""Oktober """"(1976'""","het gebruik van een binnenstad, het gebruik van de binnenstad, gebruik van een binnenstad, het gebruik van de binnenstad, persoonskenmerken, persoonskenmerken, kenmerken van de binnenstad, persoonskenmerken, gebruik van de binnenstad, gebruik van de binnen - stad, gebruik van de binnenstad",</t>
   </si>
   <si>
@@ -56,9 +53,6 @@
     <t>"(1994_Kermis_Jan_Hongarije_land_van_twee_snelheden)";Hongarije: land van de twee snelheden?',16,1994_Kermis_Jan_Hongarije_land_van_twee_snelheden," 'Martin Schluter'</t>
   </si>
   <si>
-    <t>issued</t>
-  </si>
-  <si>
     <t>thesisID</t>
   </si>
   <si>
@@ -164,9 +158,6 @@
     <t>title_cleaned</t>
   </si>
   <si>
-    <t>title_clean</t>
-  </si>
-  <si>
     <t>industrie, industriële geografie, industrieel bedrijf, industriële structuur, basisindustrie, cycletheory, groei-industrie, groeipool, herstructurering, industrialisatie, industrieel complex, industrieel klimaat, industrieel milieu, peakindustry, ontwikkelingsas, sleutelindustrie, speerpunt industrie</t>
   </si>
   <si>
@@ -222,6 +213,132 @@
   </si>
   <si>
     <t>Markeverdelingen</t>
+  </si>
+  <si>
+    <t>Ontwikkelingen in De Industriele Structuur van Zuid-West-Nederland 1945-1970, Een sociaal-geografische verkenning</t>
+  </si>
+  <si>
+    <t>Migratie: een verbetering?, Verslag van de huishoudensenquete 1973 voor het Onderzoek Middengebied Randstad</t>
+  </si>
+  <si>
+    <t>De Markeverdelingen in Zuidoost-Salland</t>
+  </si>
+  <si>
+    <t>De invloed van persoonskenmerken op verschillende vormen van gebruik van een binnenstad</t>
+  </si>
+  <si>
+    <t>Het Woongedrag in de Wijk Jutphaas-Wijkersloot - Gemeente Nieuwegein</t>
+  </si>
+  <si>
+    <t>Groeikern ook Koopkern?, Een onderzoek naar de koopgerichtheid van huishoudens in nieuwegein</t>
+  </si>
+  <si>
+    <t>Regionale Verschillen in Medische Consumptie , Een sociaal-geografische studie</t>
+  </si>
+  <si>
+    <t>Innovatiebevordering In Baden-Wuerttemberg, Op zoek naar een verklaring voor een economisch succes</t>
+  </si>
+  <si>
+    <t>Randstad en telecommunicatie</t>
+  </si>
+  <si>
+    <t>Vergrijzen in de grote stad.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Het Groene Hart van binnen naar buiten, Stemmen uit het groen , Een onderzoek naar de visie van de grootste gemeenten in het middengebied van de Randstad op de ruimtelijke ordening ervan </t>
+  </si>
+  <si>
+    <t>De Zone 16 De Julio Na Het Ham-Birf-Project., De Effecten van Buurtverbetering in El Alto, Bolivia</t>
+  </si>
+  <si>
+    <t>Winkelen Op de Uithof!, Fictie of Werkelijkheid</t>
+  </si>
+  <si>
+    <t>De Stadsregionale Bedrijventerreinenmarkt En Herstructurering: Prioriteit Of Lapmiddel?, Studie Voor de Stadsregio Eindhoven-Helmond</t>
+  </si>
+  <si>
+    <t>Hongarije: land van de twee snelheden?, De gevolgen van de transitie naar een markteconomie op de regionale economische ontwikkeling</t>
+  </si>
+  <si>
+    <t>Het PPP-project Hof/Krommestraat als voorbeeldfunctie</t>
+  </si>
+  <si>
+    <t>De Regio Stedendriehoek, Regionale ontwikkeling en de betekenis van watersystemen voor de relatie tussen stedelijk en landelijk gebied</t>
+  </si>
+  <si>
+    <t>Angstgevoelens tijdens het uitgaan</t>
+  </si>
+  <si>
+    <t>E-commerce in de binnenstad Een onderzoek naar e-commerce succes onder winkeliers in de binnenstad</t>
+  </si>
+  <si>
+    <t>author_cleaned</t>
+  </si>
+  <si>
+    <t>N.F. Abcouwer</t>
+  </si>
+  <si>
+    <t>Jan Jaap Harts</t>
+  </si>
+  <si>
+    <t>F.W.J Scholten</t>
+  </si>
+  <si>
+    <t>M.J. Boskamp</t>
+  </si>
+  <si>
+    <t>Rolf v. Acquoy, Wil Anker, Dorothe Bloks, Frank Gubbels, Rolf Hunink, Joep Jilesen, Oda v.d. Kemp, Dick Korenhof, Wim v.d. Maas, Roel de Mink, Jan Mulder, Lody Smeets, Ben Steur, Monica Thung, Saskia Vleer</t>
+  </si>
+  <si>
+    <t>Henk Baten</t>
+  </si>
+  <si>
+    <t>A. G. M. Van Elzakker</t>
+  </si>
+  <si>
+    <t>Robert Hassink</t>
+  </si>
+  <si>
+    <t>Jeroen de Roos</t>
+  </si>
+  <si>
+    <t>Frank Studulski, Hidde Toet</t>
+  </si>
+  <si>
+    <t>M . van Noordenne</t>
+  </si>
+  <si>
+    <t>Paul van Beijnum, Ronald H. Kranenburg</t>
+  </si>
+  <si>
+    <t>Eefke Langendonk</t>
+  </si>
+  <si>
+    <t>Emmy Hessels, Jeroen Smit</t>
+  </si>
+  <si>
+    <t>Jan Kennis, Martin Schluter</t>
+  </si>
+  <si>
+    <t>Martin Slabbertje</t>
+  </si>
+  <si>
+    <t>Klaske W. Ypma</t>
+  </si>
+  <si>
+    <t>Frank de Beer</t>
+  </si>
+  <si>
+    <t>Stefan de Jong</t>
+  </si>
+  <si>
+    <t>issued_cleaned</t>
+  </si>
+  <si>
+    <t>De Shell-Raffinaderij Op Curacao; Haar Sociaal-Economische Effecten</t>
+  </si>
+  <si>
+    <t>Willy Dwarkasing</t>
   </si>
 </sst>
 </file>
@@ -729,13 +846,15 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1111,317 +1230,496 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5EE7E4C-92F7-4004-A116-4A0ED83F8F04}">
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.6328125" customWidth="1"/>
-    <col min="7" max="7" width="10.90625" customWidth="1"/>
-    <col min="8" max="8" width="67.36328125" style="2" customWidth="1"/>
-    <col min="9" max="9" width="58.6328125" customWidth="1"/>
+    <col min="1" max="1" width="66.6328125" customWidth="1"/>
+    <col min="4" max="4" width="106.1796875" customWidth="1"/>
+    <col min="5" max="5" width="33.7265625" customWidth="1"/>
+    <col min="6" max="6" width="28.6328125" style="6" customWidth="1"/>
+    <col min="7" max="7" width="67.36328125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="58.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E1" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="G1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C1" t="s">
+      <c r="H1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E1" t="s">
-        <v>46</v>
-      </c>
-      <c r="F1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
-      <c r="H2" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="I2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="D2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E2" t="s">
+        <v>84</v>
+      </c>
+      <c r="F2" s="6">
+        <v>1971</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="H2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B3">
         <v>2</v>
       </c>
-      <c r="H3" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="I3" t="s">
+      <c r="D3" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="E3" t="s">
+        <v>85</v>
+      </c>
+      <c r="F3" s="6">
+        <v>1974</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B4" s="1">
         <v>3</v>
       </c>
-      <c r="H4" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="I4" s="1" t="s">
+      <c r="D4" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="E4" t="s">
+        <v>86</v>
+      </c>
+      <c r="F4" s="6">
+        <v>1974</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B5">
         <v>4</v>
       </c>
-      <c r="H5" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="I5" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="D5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E5" t="s">
+        <v>87</v>
+      </c>
+      <c r="F5" s="6">
+        <v>1976</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="H5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B6">
         <v>5</v>
       </c>
-      <c r="H6" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="I6" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="D6" t="s">
+        <v>68</v>
+      </c>
+      <c r="E6" t="s">
+        <v>88</v>
+      </c>
+      <c r="F6" s="6">
+        <v>1979</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H6" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B7">
         <v>6</v>
       </c>
-      <c r="H7" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="I7" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="D7" t="s">
+        <v>69</v>
+      </c>
+      <c r="E7" t="s">
+        <v>89</v>
+      </c>
+      <c r="F7" s="6">
+        <v>1982</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B8">
         <v>7</v>
       </c>
-      <c r="H8" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="I8" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="D8" t="s">
+        <v>70</v>
+      </c>
+      <c r="E8" t="s">
+        <v>90</v>
+      </c>
+      <c r="F8" s="6">
+        <v>1984</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="H8" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B9">
         <v>8</v>
       </c>
-      <c r="H9" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I9" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="D9" t="s">
+        <v>104</v>
+      </c>
+      <c r="E9" t="s">
+        <v>105</v>
+      </c>
+      <c r="F9" s="6">
+        <v>1985</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B10">
         <v>9</v>
       </c>
-      <c r="H10" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="I10" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="D10" t="s">
+        <v>71</v>
+      </c>
+      <c r="E10" t="s">
+        <v>91</v>
+      </c>
+      <c r="F10" s="6">
+        <v>1988</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H10" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B11">
         <v>10</v>
       </c>
-      <c r="H11" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="I11" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="D11" t="s">
+        <v>72</v>
+      </c>
+      <c r="E11" t="s">
+        <v>92</v>
+      </c>
+      <c r="F11" s="6">
+        <v>1988</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H11" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B12">
         <v>11</v>
       </c>
-      <c r="H12" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="I12" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="D12" t="s">
+        <v>73</v>
+      </c>
+      <c r="E12" t="s">
+        <v>93</v>
+      </c>
+      <c r="F12" s="6">
+        <v>1988</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="H12" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B13">
         <v>12</v>
       </c>
-      <c r="H13" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="I13" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D13" t="s">
+        <v>74</v>
+      </c>
+      <c r="E13" t="s">
+        <v>94</v>
+      </c>
+      <c r="F13" s="6">
+        <v>1989</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="H13" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B14" s="1">
         <v>13</v>
       </c>
-      <c r="H14" s="2"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="D14" t="s">
+        <v>75</v>
+      </c>
+      <c r="E14" t="s">
+        <v>95</v>
+      </c>
+      <c r="F14" s="7">
+        <v>1993</v>
+      </c>
+      <c r="G14" s="2"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B15">
         <v>14</v>
       </c>
-      <c r="H15" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="I15" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="D15" t="s">
+        <v>76</v>
+      </c>
+      <c r="E15" t="s">
+        <v>96</v>
+      </c>
+      <c r="F15" s="6">
+        <v>1993</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H15" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B16">
         <v>15</v>
       </c>
-      <c r="H16" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="I16" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="D16" t="s">
+        <v>77</v>
+      </c>
+      <c r="E16" t="s">
+        <v>97</v>
+      </c>
+      <c r="F16" s="6">
+        <v>1994</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H16" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B17">
         <v>16</v>
       </c>
+      <c r="D17" t="s">
+        <v>78</v>
+      </c>
+      <c r="E17" t="s">
+        <v>98</v>
+      </c>
+      <c r="F17" s="6">
+        <v>1994</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>39</v>
+      </c>
       <c r="H17" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="I17" s="4" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B18">
         <v>17</v>
       </c>
-      <c r="H18" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="I18" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="D18" t="s">
+        <v>79</v>
+      </c>
+      <c r="E18" t="s">
+        <v>99</v>
+      </c>
+      <c r="F18" s="6">
+        <v>1994</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H18" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B19">
         <v>18</v>
       </c>
-      <c r="H19" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="I19" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="D19" t="s">
+        <v>80</v>
+      </c>
+      <c r="E19" t="s">
+        <v>100</v>
+      </c>
+      <c r="F19" s="6">
+        <v>1995</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="H19" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B20">
         <v>19</v>
       </c>
-      <c r="H20" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="I20" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="D20" t="s">
+        <v>81</v>
+      </c>
+      <c r="E20" t="s">
+        <v>101</v>
+      </c>
+      <c r="F20" s="6">
+        <v>2007</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="H20" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B21">
         <v>20</v>
       </c>
-      <c r="H21" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="I21" t="s">
-        <v>51</v>
+      <c r="D21" t="s">
+        <v>82</v>
+      </c>
+      <c r="E21" t="s">
+        <v>102</v>
+      </c>
+      <c r="F21" s="6">
+        <v>2007</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="H21" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add cleaned up spatials
</commit_message>
<xml_diff>
--- a/code/data_cleaning/annotations_summary_manually_edited.xlsx
+++ b/code/data_cleaning/annotations_summary_manually_edited.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\5298954\Documents\Github_Repos\GIMA_thesis\code\data_cleaning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{399BBC61-2D36-4DE3-A9AD-2F6D739FF93B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4589BE73-2ABD-4DE8-9DE5-FA92403366EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-9540" windowWidth="29040" windowHeight="15720" xr2:uid="{1CC9DFF3-CCD0-41B0-B0A8-07B4A468A7A4}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="148">
   <si>
     <t>File</t>
   </si>
@@ -339,6 +339,132 @@
   </si>
   <si>
     <t>Willy Dwarkasing</t>
+  </si>
+  <si>
+    <t>spatial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spatial_cleaned </t>
+  </si>
+  <si>
+    <t>Rijnmond', 'Rijnmond', 'Rijnmond', 'Rijnmond', 'Rijnmond', 'Rijnmond-Zuid-West Nederland', 'Rijnmond', 'Zuid-West Nederland', 'Rijnmond', 'Rijnmond', 'Rotterdam ( Rijnmond )', 'Zuidelijke Randstad'</t>
+  </si>
+  <si>
+    <t>Rijnmond, Rijnmond-Zuid-West Nederland, Zuid-West Nederland, Rotterdam, Zuidelijke Randstad</t>
+  </si>
+  <si>
+    <t>Middengebied Randstad</t>
+  </si>
+  <si>
+    <t>Amersfoortse, Amersfoort, Hoevelaken, Leusden, Soest, Eemnes, Bunschoten, Nijkerk</t>
+  </si>
+  <si>
+    <t>Jutphaas-Wijkersloot</t>
+  </si>
+  <si>
+    <t>Nieuwegein, De negen woonwijken van Nieuwegein</t>
+  </si>
+  <si>
+    <t>Nederland</t>
+  </si>
+  <si>
+    <t>Curaçao, Nederlandse Antillen, Willemstad</t>
+  </si>
+  <si>
+    <t>Baden-Württemberg</t>
+  </si>
+  <si>
+    <t>Vier grote steden, Amsterdam, Rotterdam, Den Haag, Utrecht</t>
+  </si>
+  <si>
+    <t>Groene Hart, Het gebied tussen de vier grote steden Amsterdam, Den Haag, Rotterdam, Utrecht, Middengebied van de Randstad, Het niet verstedelijkte gebied bij die stad, Een gebied overeenkomstig het Open Middengebied Noord, Utrechts Weidegebied, Noordelijke veenstreek in Zuid-Holland, Rijnstreek Zuid-Holland, Gouda en omstreken, Krimpenerwaard, Benthuizen, Bleiswijk, Moerkapelle, Nieuwerkerk a/d IJssel, Zevenhuizen, Vinkeveen, Waverveen, IJsselstein, Gouda, Alphen a/d Rijn, Woerden, Waddinxveen, Bodegraven, De Ronde Venen, Schoonhoven</t>
+  </si>
+  <si>
+    <t>De Uithof, Utrecht, Universiteit Utrecht</t>
+  </si>
+  <si>
+    <t>Stadsregio Eindhoven-Helmond, Veldhoven, Eindhoven, Best, Geldrop, Nuenen, Son en Breugel, Waalre, Aarle-Rixtel, Mierlo, Helmond</t>
+  </si>
+  <si>
+    <t>Hongarije</t>
+  </si>
+  <si>
+    <t>Hof/Krommestraat in Amersfoort, Langestraat northeast of the Joriskerk, Hof/Krommestraat area</t>
+  </si>
+  <si>
+    <t>Apeldoorn, Deventer, Zutphen, Regio Stedendriehoek, Gewest Midden-IJssel, Oost-Veluwe, Overijssel, Gelderland</t>
+  </si>
+  <si>
+    <t>Het Caterplein, De noordzijde van de Hoofdstraat en het Beekpark, Beekpark, Apeldoorn</t>
+  </si>
+  <si>
+    <t>Amersfoort, Almere, Alkmaar, Haarlem, Hilversum, Purmerend, Utrecht, Veenendaal</t>
+  </si>
+  <si>
+    <t>El Alto, Bolivia, La Paz, De zone 16 de Julio</t>
+  </si>
+  <si>
+    <t>'het Middengebied Randstad', 'Middengebied Randstad', 'middengebied', 'Middengebied Randstad'</t>
+  </si>
+  <si>
+    <t>'Amersfoortse', 'Amersfoort', 'Amersfoort', 'Amersfoort', 'Amersfoort', 'Amersfoort', 'Amersfoort', 'Hoevelaken', 'Leus - den', 'Soest', 'Eemnes', 'Bunschoten', 'Nijkerk'</t>
+  </si>
+  <si>
+    <t>'Jutphaas - Wijkersloot', 'Jutphaas-Wijkersloot', 'Jutphaas-Wijkersloot', 'Jutphaas-Wijkersloot'</t>
+  </si>
+  <si>
+    <t>'Nieuwegein', 'Nieuwegein', 'Nieuwegein', 'Nieuwegein', 'Nieuwegein', 'de negen woonwijken van Nieuwegein'</t>
+  </si>
+  <si>
+    <t>'Nederland', 'Nederlandse verzorgingsstaat', 'Nederlandse verzorgingsstaat', 'Nederlandse gezondheidszorgapparaat'</t>
+  </si>
+  <si>
+    <t>'Curacao', 'Curacao', 'Nederlandse Antillen', 'Nederlandse Antillen', 'Curacao', 'Curacao', 'Curacao', 'Nederlandse Antillen', 'Willemstad'</t>
+  </si>
+  <si>
+    <t>'Baden-Wurttemberg', 'Baden-Wurttemberg', 'deelstaat Baden-Wurttemberg', 'Baden-Wurttemberg'</t>
+  </si>
+  <si>
+    <t>'gemeenten Amsterdam , Den Haag en Rotterdam , bij de provincie Utrecht', 'PTT-T distrikten Amsterdam , Den Haag , Rotterdam en Utrecht', 'de vier grote Randstadâ€”steden', 'de gemeenten Amsterdam , Den Haag , Rotter - dam en Utrecht', 'Randstad', 'Nederland', 'Randstad', 'Randstad', 'Nederland', 'Randstad'</t>
+  </si>
+  <si>
+    <t>'grote steden', 'vier grote steden', 'Amsterdam', 'Rotterdam', 'Den Haag', 'Utrecht', 'vier grote steden', 'Amsterdam', 'Den Haag', 'Rotterdam', 'Utrecht'</t>
+  </si>
+  <si>
+    <t>'Groene Hart', 'Groene Hart', 'Groene Hart', 'Groene Hart', 'Groene Hart', 'Groene Hart', 'Groene Hart', 'het gebied tussen de vier grote steden , Amsterdam , Den Haag , Rotterdam en Utrecht', 'middenge - bied van de Randstad', 'het niet verstedelijkte gebied bij die stad', ""een gebied overeenkomstig het ' Open Middengebied Noord '"", 'Utrechts Weidegebied', 'Noordelijke veenstreek in Zuid-Holland', 'Rijnstreek Zuid-Hol - land', 'Gouda en omstreken', 'Krimpenerwaard', 'Benthuizen', 'Bleiswijk', 'Moerkapelle', 'Nieuwerkerk a / d Ussel', 'Zevenhuizen', 'Vinkeveen', 'Waverveen', 'Usselstein', 'Gouda', 'Alphen a / d Rijn', 'Woerden', 'Waddinxveen', 'Ussel - stein', 'Nieuwerkerk a / d Ussel', 'Bodegraven', 'De Ronde Venen', 'Schoonhoven'</t>
+  </si>
+  <si>
+    <t>'El Alto , Bolivia .', 'Bolivia', 'La Paz', 'La Paz', 'El Alto', 'Bolivia', 'El Alto', 'El Alto', 'El Alto', 'La Paz', 'El Alto', 'de zone 16 de Julio', 'El Alto', 'zone 16 de Julio', 'zone 16 de Julio', 'zone 16 de Julio', 'longitudinale analyse', 'zone 16 de Julio .', 'zone 16 de Julio'</t>
+  </si>
+  <si>
+    <t>'De Uithof', 'Utrecht .', 'Universiteit Utrecht', 'Utrecht', 'Uithof', 'Uithof', 'Uithof', 'Uithof', 'Uithof', 'Uithof', 'Uithof'</t>
+  </si>
+  <si>
+    <t>'Stadsregio Eindhoven-Helmond', 'stadsregio Eindhoven-Helmond', 'Veldhoven', 'Eindhoven', 'Eindhoven / Helmond', 'stadsregio Eindhoven-Helmond', 'stadsregio Eindhoven-Helmond', 'Best', 'Geldrop', 'Nuenen', 'Son en Breugel', 'Veldhoven', 'Waalre', 'Aarle-Rixtel', 'Mierlo', 'stadsregio Eindhoven-Helmond', 'Eindhoven', 'Helmond'</t>
+  </si>
+  <si>
+    <t>'Hungary', 'Hungary', 'Hungary', 'Hungary', 'Hungary', 'Hongarije', 'Hongarije', 'Hongarije', 'Hongarije', 'Hongarije'</t>
+  </si>
+  <si>
+    <t>'het winkel / uitgaansgebied Hof / Krommestraat in Amersfoort', 'Langestraat ten noordoosten van de Joriskerk', 'in het gebied Hof / Krommestraat', 'gebied Hof / Krommestraat'</t>
+  </si>
+  <si>
+    <t>'Apeldoorn', 'Deventer', 'Zutphen', 'Regio Stedendriehoek', 'Regio Stedendriehoek', 'Gewest Midden-Ussel ( GMU )', 'Samenwerkingsorgaan Oost-Veluwe ( SOV )', 'Regio Stedendriehoek', 'Overijssel', 'Gelderland', 'Apeldoorn', 'Deventer', 'Zutphen', 'Regio Stedendriehoek'</t>
+  </si>
+  <si>
+    <t>'gemeente Apeldoorn', 'het Caterplein', 'het Caterplein', 'het Caterplein', 'de noordzijde van de Hoofdstraat en het Beekpark', 'een park als een straat met de naam Beekpark', 'in Apeldoorn', 'het Caterplein in Apeldoorn'</t>
+  </si>
+  <si>
+    <t>'Amersfoort', 'Almere', 'Alkmaar', 'Haarlem', 'Hilversum', 'Purmerend', 'Utrecht', 'Veenendaal', 'Alkmaar', 'Almere', 'Amersfoort', 'Haarlem', 'Hilversum ,', 'Purmerend', 'Utrecht', 'Veenendaal'</t>
+  </si>
+  <si>
+    <t>Oost-nederland', 'luid-l.Hand', 'Hellendoorn', 'Duttenberg', ""1 ' Toetsele"", 'Daarle', 'Zuid-Salland', 'Zuid-Salland', 'Zuid-Salland', 'Zuid-Salland', 'Zuid-Salland', 'Luttenborg', 'Hellen - doorn', 'IToetsele', 'Daarle', 'Luttenborg', 'Ilellendoornso', 'IToetselor Derg', 'Daarle', 'Scharlonbelt', 'Hollendoorn'</t>
+  </si>
+  <si>
+    <t>Oost-Nederland, Hellendoorn, Luttenberg, Daarle, Zuid-Salland, Noetsele, Noetselerberg, Scharlonbelt</t>
+  </si>
+  <si>
+    <t>Amsterdam, Den Haag, Rotterdam, PTT-T districten Amsterdam  Den Haag Rotterdam, de vier grote Randstadsteden, Utrecht, Nederland, Randstad</t>
   </si>
 </sst>
 </file>
@@ -846,7 +972,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
@@ -855,6 +981,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1230,18 +1360,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5EE7E4C-92F7-4004-A116-4A0ED83F8F04}">
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="66.6328125" customWidth="1"/>
-    <col min="4" max="4" width="106.1796875" customWidth="1"/>
-    <col min="5" max="5" width="33.7265625" customWidth="1"/>
-    <col min="6" max="6" width="28.6328125" style="6" customWidth="1"/>
-    <col min="7" max="7" width="67.36328125" style="2" customWidth="1"/>
-    <col min="8" max="8" width="58.6328125" customWidth="1"/>
+    <col min="3" max="3" width="0" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="106.1796875" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="33.7265625" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="28.6328125" style="6" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="67.36328125" style="2" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="58.6328125" hidden="1" customWidth="1"/>
+    <col min="9" max="10" width="58.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1266,8 +1398,14 @@
       <c r="H1" s="3" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I1" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -1289,8 +1427,14 @@
       <c r="H2" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I2" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="J2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>22</v>
       </c>
@@ -1312,8 +1456,14 @@
       <c r="H3" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="I3" t="s">
+        <v>127</v>
+      </c>
+      <c r="J3" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>19</v>
       </c>
@@ -1335,8 +1485,14 @@
       <c r="H4" s="1" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I4" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -1358,8 +1514,14 @@
       <c r="H5" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I5" t="s">
+        <v>128</v>
+      </c>
+      <c r="J5" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1381,8 +1543,14 @@
       <c r="H6" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I6" t="s">
+        <v>129</v>
+      </c>
+      <c r="J6" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>2</v>
       </c>
@@ -1404,8 +1572,14 @@
       <c r="H7" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I7" t="s">
+        <v>130</v>
+      </c>
+      <c r="J7" s="10" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -1427,8 +1601,14 @@
       <c r="H8" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I8" t="s">
+        <v>131</v>
+      </c>
+      <c r="J8" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -1450,8 +1630,14 @@
       <c r="H9" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I9" t="s">
+        <v>132</v>
+      </c>
+      <c r="J9" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -1473,8 +1659,14 @@
       <c r="H10" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I10" t="s">
+        <v>133</v>
+      </c>
+      <c r="J10" s="10" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -1496,8 +1688,14 @@
       <c r="H11" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I11" t="s">
+        <v>134</v>
+      </c>
+      <c r="J11" s="11" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -1519,8 +1717,14 @@
       <c r="H12" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I12" t="s">
+        <v>135</v>
+      </c>
+      <c r="J12" s="10" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>5</v>
       </c>
@@ -1542,8 +1746,14 @@
       <c r="H13" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="I13" t="s">
+        <v>136</v>
+      </c>
+      <c r="J13" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>6</v>
       </c>
@@ -1560,8 +1770,14 @@
         <v>1993</v>
       </c>
       <c r="G14" s="2"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I14" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>7</v>
       </c>
@@ -1583,8 +1799,14 @@
       <c r="H15" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I15" t="s">
+        <v>138</v>
+      </c>
+      <c r="J15" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>8</v>
       </c>
@@ -1606,8 +1828,14 @@
       <c r="H16" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I16" t="s">
+        <v>139</v>
+      </c>
+      <c r="J16" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>9</v>
       </c>
@@ -1626,11 +1854,17 @@
       <c r="G17" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="H17" s="4" t="s">
+      <c r="H17" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I17" t="s">
+        <v>140</v>
+      </c>
+      <c r="J17" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>26</v>
       </c>
@@ -1652,8 +1886,14 @@
       <c r="H18" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I18" t="s">
+        <v>141</v>
+      </c>
+      <c r="J18" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>25</v>
       </c>
@@ -1675,8 +1915,14 @@
       <c r="H19" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I19" t="s">
+        <v>142</v>
+      </c>
+      <c r="J19" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>24</v>
       </c>
@@ -1698,8 +1944,14 @@
       <c r="H20" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I20" t="s">
+        <v>143</v>
+      </c>
+      <c r="J20" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>23</v>
       </c>
@@ -1720,6 +1972,12 @@
       </c>
       <c r="H21" t="s">
         <v>48</v>
+      </c>
+      <c r="I21" t="s">
+        <v>144</v>
+      </c>
+      <c r="J21" t="s">
+        <v>125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>